<commit_message>
Cleaned the code and folders
</commit_message>
<xml_diff>
--- a/results/tables/Summary_of_analysises_torress_PP.xlsx
+++ b/results/tables/Summary_of_analysises_torress_PP.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="565">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -1586,45 +1586,78 @@
     <t xml:space="preserve">Variable_to_explain</t>
   </si>
   <si>
-    <t xml:space="preserve">OR_CI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p_value</t>
+    <t xml:space="preserve">OR_CI_not_adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_value_1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OR_CI_adjusted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_value_2</t>
   </si>
   <si>
     <t xml:space="preserve">0.22 (0.07 - 0.72)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.13 (0.03 - 0.55)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.76 (0.16 - 3.65)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.49 (0.06 - 4.06)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.68 (0.11 - 4.32)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.24 (0.01 - 4.84)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.51 (0.04 - 5.94)</t>
   </si>
   <si>
+    <t xml:space="preserve">0 (0 - 126728.6)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1 (0 - Inf)</t>
   </si>
   <si>
     <t xml:space="preserve">0.06 (0.01 - 0.51)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.04 (0 - 0.35)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.11 (0.01 - 0.96)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.06 (0.01 - 0.63)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.19 (0.02 - 1.75)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.13 (0.01 - 1.4)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.25 (0.03 - 2.33)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.14 (0.01 - 1.71)</t>
+  </si>
+  <si>
     <t xml:space="preserve">0 (0 - Inf)</t>
   </si>
   <si>
     <t xml:space="preserve">0.41 (0.1 - 1.71)</t>
   </si>
   <si>
+    <t xml:space="preserve">0.07 (0.01 - 0.91)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Time</t>
   </si>
   <si>
@@ -1634,13 +1667,7 @@
     <t xml:space="preserve">HR_CI_not_adjusted</t>
   </si>
   <si>
-    <t xml:space="preserve">p_value_1</t>
-  </si>
-  <si>
     <t xml:space="preserve">HR_CI_adjusted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">p_value_2</t>
   </si>
   <si>
     <t xml:space="preserve">ph_test_p_value</t>
@@ -5493,16 +5520,28 @@
       <c r="C1" t="s">
         <v>523</v>
       </c>
+      <c r="D1" t="s">
+        <v>524</v>
+      </c>
+      <c r="E1" t="s">
+        <v>525</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
         <v>484</v>
       </c>
       <c r="B2" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="C2" t="n">
         <v>0.012979069543786</v>
+      </c>
+      <c r="D2" t="s">
+        <v>527</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0061679761801535</v>
       </c>
     </row>
     <row r="3">
@@ -5510,10 +5549,16 @@
         <v>475</v>
       </c>
       <c r="B3" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="C3" t="n">
         <v>0.73393319381818</v>
+      </c>
+      <c r="D3" t="s">
+        <v>529</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.504979245344167</v>
       </c>
     </row>
     <row r="4">
@@ -5521,10 +5566,16 @@
         <v>422</v>
       </c>
       <c r="B4" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="C4" t="n">
         <v>0.679335051092047</v>
+      </c>
+      <c r="D4" t="s">
+        <v>531</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.349278237240908</v>
       </c>
     </row>
     <row r="5">
@@ -5532,10 +5583,16 @@
         <v>430</v>
       </c>
       <c r="B5" t="s">
-        <v>527</v>
+        <v>532</v>
       </c>
       <c r="C5" t="n">
         <v>0.587292264203728</v>
+      </c>
+      <c r="D5" t="s">
+        <v>533</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.203728912203729</v>
       </c>
     </row>
     <row r="6">
@@ -5543,9 +5600,15 @@
         <v>436</v>
       </c>
       <c r="B6" t="s">
-        <v>528</v>
+        <v>534</v>
       </c>
       <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>534</v>
+      </c>
+      <c r="E6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5554,10 +5617,16 @@
         <v>478</v>
       </c>
       <c r="B7" t="s">
-        <v>529</v>
+        <v>535</v>
       </c>
       <c r="C7" t="n">
         <v>0.0100695377057599</v>
+      </c>
+      <c r="D7" t="s">
+        <v>536</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.00496210635213492</v>
       </c>
     </row>
     <row r="8">
@@ -5565,10 +5634,16 @@
         <v>446</v>
       </c>
       <c r="B8" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
       <c r="C8" t="n">
         <v>0.0460987014737764</v>
+      </c>
+      <c r="D8" t="s">
+        <v>538</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.0194506565283575</v>
       </c>
     </row>
     <row r="9">
@@ -5576,10 +5651,16 @@
         <v>450</v>
       </c>
       <c r="B9" t="s">
-        <v>531</v>
+        <v>539</v>
       </c>
       <c r="C9" t="n">
         <v>0.141597467275331</v>
+      </c>
+      <c r="D9" t="s">
+        <v>540</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.0915350022488128</v>
       </c>
     </row>
     <row r="10">
@@ -5587,10 +5668,16 @@
         <v>456</v>
       </c>
       <c r="B10" t="s">
-        <v>532</v>
+        <v>541</v>
       </c>
       <c r="C10" t="n">
         <v>0.218254650658311</v>
+      </c>
+      <c r="D10" t="s">
+        <v>542</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.122220618920276</v>
       </c>
     </row>
     <row r="11">
@@ -5598,10 +5685,16 @@
         <v>459</v>
       </c>
       <c r="B11" t="s">
-        <v>533</v>
+        <v>543</v>
       </c>
       <c r="C11" t="n">
         <v>0.994012655180835</v>
+      </c>
+      <c r="D11" t="s">
+        <v>543</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.98946136131057</v>
       </c>
     </row>
     <row r="12">
@@ -5609,10 +5702,16 @@
         <v>463</v>
       </c>
       <c r="B12" t="s">
-        <v>534</v>
+        <v>544</v>
       </c>
       <c r="C12" t="n">
         <v>0.219565394472554</v>
+      </c>
+      <c r="D12" t="s">
+        <v>545</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0426554316032057</v>
       </c>
     </row>
   </sheetData>
@@ -5628,28 +5727,28 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>535</v>
+        <v>546</v>
       </c>
       <c r="B1" t="s">
-        <v>536</v>
+        <v>547</v>
       </c>
       <c r="C1" t="s">
-        <v>537</v>
+        <v>548</v>
       </c>
       <c r="D1" t="s">
-        <v>538</v>
+        <v>523</v>
       </c>
       <c r="E1" t="s">
-        <v>539</v>
+        <v>549</v>
       </c>
       <c r="F1" t="s">
-        <v>540</v>
+        <v>525</v>
       </c>
       <c r="G1" t="s">
-        <v>541</v>
+        <v>550</v>
       </c>
       <c r="H1" t="s">
-        <v>542</v>
+        <v>551</v>
       </c>
     </row>
     <row r="2">
@@ -5657,16 +5756,16 @@
         <v>185</v>
       </c>
       <c r="B2" t="s">
-        <v>543</v>
+        <v>552</v>
       </c>
       <c r="C2" t="s">
-        <v>544</v>
+        <v>553</v>
       </c>
       <c r="D2" t="n">
         <v>0.0278381911228222</v>
       </c>
       <c r="E2" t="s">
-        <v>545</v>
+        <v>554</v>
       </c>
       <c r="F2" t="n">
         <v>0.080008655112598</v>
@@ -5675,7 +5774,7 @@
         <v>0.198</v>
       </c>
       <c r="H2" t="s">
-        <v>546</v>
+        <v>555</v>
       </c>
     </row>
     <row r="3">
@@ -5683,16 +5782,16 @@
         <v>158</v>
       </c>
       <c r="B3" t="s">
-        <v>547</v>
+        <v>556</v>
       </c>
       <c r="C3" t="s">
-        <v>548</v>
+        <v>557</v>
       </c>
       <c r="D3" t="n">
         <v>0.959420406674248</v>
       </c>
       <c r="E3" t="s">
-        <v>549</v>
+        <v>558</v>
       </c>
       <c r="F3" t="n">
         <v>0.994342116239634</v>
@@ -5701,7 +5800,7 @@
         <v>0.487</v>
       </c>
       <c r="H3" t="s">
-        <v>546</v>
+        <v>555</v>
       </c>
     </row>
     <row r="4">
@@ -5709,16 +5808,16 @@
         <v>168</v>
       </c>
       <c r="B4" t="s">
-        <v>550</v>
+        <v>559</v>
       </c>
       <c r="C4" t="s">
-        <v>551</v>
+        <v>560</v>
       </c>
       <c r="D4" t="n">
         <v>0.498437991931803</v>
       </c>
       <c r="E4" t="s">
-        <v>552</v>
+        <v>561</v>
       </c>
       <c r="F4" t="n">
         <v>0.868793120079614</v>
@@ -5727,7 +5826,7 @@
         <v>0.315</v>
       </c>
       <c r="H4" t="s">
-        <v>546</v>
+        <v>555</v>
       </c>
     </row>
     <row r="5">
@@ -5735,16 +5834,16 @@
         <v>177</v>
       </c>
       <c r="B5" t="s">
-        <v>553</v>
+        <v>562</v>
       </c>
       <c r="C5" t="s">
-        <v>554</v>
+        <v>563</v>
       </c>
       <c r="D5" t="n">
         <v>0.877089351112259</v>
       </c>
       <c r="E5" t="s">
-        <v>555</v>
+        <v>564</v>
       </c>
       <c r="F5" t="n">
         <v>0.420601046900591</v>
@@ -5753,7 +5852,7 @@
         <v>0.084</v>
       </c>
       <c r="H5" t="s">
-        <v>546</v>
+        <v>555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>